<commit_message>
docs: add literature notes and evidence-backed survey
</commit_message>
<xml_diff>
--- a/data/pyscf_quantum_chemistry_visualization_research_2026-07-19.xlsx
+++ b/data/pyscf_quantum_chemistry_visualization_research_2026-07-19.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="Rd20d26b660f34ffb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心文献" sheetId="2" r:id="Rc26356d27f45482d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="软件矩阵" sheetId="3" r:id="R09beb7550d8444a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问卷题库" sheetId="4" r:id="Rf88f37b138614d25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="验证矩阵" sheetId="5" r:id="R89da4d2e75a842d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R409b118de44e494d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心文献" sheetId="2" r:id="R890775931842497d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="软件矩阵" sheetId="3" r:id="R85762cda090344d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问卷题库" sheetId="4" r:id="R673f7b00a66847bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="验证矩阵" sheetId="5" r:id="R397611d2db8a4b14"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -626,7 +626,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd5f7c5d4c04b49c3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R96f7aa38fdbc440e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -893,7 +893,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="12" t="str">
-        <x:v>检索与整理日期：2026-07-19｜证据分层：同行评议、官方资料、公开技术讨论、社区调查</x:v>
+        <x:v>检索与整理：2026-07-19；全文笔记与问卷依据更新：2026-07-20｜证据分层：同行评议、官方资料、公开技术讨论、社区调查</x:v>
       </x:c>
       <x:c r="B2" s="12"/>
       <x:c r="C2" s="12"/>
@@ -923,7 +923,7 @@
         <x:v>方向判断</x:v>
       </x:c>
       <x:c r="C5" s="28" t="str">
-        <x:v>值得继续，但不能定位成“PySCF专用cube→VDB转换器”。已有Den2Obj和Molecular Blender等先例。可防御价值应是：引擎无关、物理语义正确、可验证、可复现、适合大体数据和动画的完整工作流。</x:v>
+        <x:v>Blender量子化学/科学可视化已有Rhorix、QMBlender、BlendMol和Digichem先例；科学元数据、误差量化和跨后端可追溯性是待问卷验证的差异化假设。证据：data/literature-notes/README.md</x:v>
       </x:c>
       <x:c r="E5" s="63" t="str">
         <x:v>文献条目</x:v>
@@ -939,10 +939,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="55" t="str">
-        <x:v>PySCF认可度</x:v>
+        <x:v>PySCF定位</x:v>
       </x:c>
       <x:c r="C6" s="30" t="str">
-        <x:v>PySCF已有高质量软件论文、活跃版本、广泛方法覆盖、周期体系和GPU/工业应用证据。它在方法开发、自动化和Python生态中的可信度很强；但传统GUI、原生Windows和部分任务性能不必然优于Gaussian/ORCA。</x:v>
+        <x:v>PySCF的Python宿主语言、可组合对象、插件式方法开发和分子—周期覆盖由框架与更新论文直接说明；适合作为首个深度后端是工程选择。证据：data/literature-notes/01-pyscf-core/sun_p_2018.md；sun_recent_2020.md</x:v>
       </x:c>
       <x:c r="E6" s="70" t="n">
         <x:v>72</x:v>
@@ -958,10 +958,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="55" t="str">
-        <x:v>与Gaussian差异</x:v>
+        <x:v>比较边界</x:v>
       </x:c>
       <x:c r="C7" s="30" t="str">
-        <x:v>Gaussian是成熟商业集成程序包；PySCF是开放Python框架/库。前者强调现成流程、培训和商业支持，后者强调透明、可修改、可嵌入和可扩展。准确度主要由计算协议决定，不由品牌单独决定。</x:v>
+        <x:v>现有61篇笔记没有统一控制条件下的PySCF—Gaussian全面比较，因此不做单一准确度或采用率排名。证据边界：docs/research/pyscf_quantum_chemistry_visualization_research_2026-07-19.md</x:v>
       </x:c>
       <x:c r="E7" s="70"/>
       <x:c r="F7" s="70"/>
@@ -973,10 +973,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="55" t="str">
-        <x:v>证明策略</x:v>
+        <x:v>证据策略</x:v>
       </x:c>
       <x:c r="C8" s="30" t="str">
-        <x:v>不要用GitHub星标或单一引用量证明“行业认可”。应组合：同行评议软件论文、独立/跨代码基准、版本与测试成熟度、生态互操作、真实用户/行业案例、分层问卷和访谈。</x:v>
+        <x:v>科学可信度应结合同行评议、公开协议、跨程序基准、版本/默认值记录和回归测试，不以引用量或GitHub指标单独代替。证据：data/literature-notes/03-numerical-reliability/；04-interoperability-workflows/</x:v>
       </x:c>
       <x:c r="E8" s="70"/>
       <x:c r="F8" s="70"/>
@@ -991,7 +991,7 @@
         <x:v>下一步</x:v>
       </x:c>
       <x:c r="C9" s="33" t="str">
-        <x:v>关键全文已核验，问卷进入10–15人认知预测试；产品路线先完成多格式与科学完整性验证，再扩展多引擎适配和高级场类型。</x:v>
+        <x:v>61篇全文阅读笔记已与2026-07-20 BibTeX按DOI一一匹配；问卷保持30题、预计12–15分钟，下一步进行10–15人认知预测试。索引：data/literature-notes/README.md</x:v>
       </x:c>
       <x:c r="E9" s="63" t="str">
         <x:v>软件矩阵</x:v>
@@ -1211,7 +1211,7 @@
     <x:mergeCell ref="A25:H25"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7eb9d65a9f584435"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a2af5c5014048f8"/>
 </x:worksheet>
 </file>
 
@@ -5150,7 +5150,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38ca4bcf04d74bb3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77c7171ed7e24ca1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6234,7 +6234,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d93ea5943694a0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddbd0e09eedc495a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6539,7 +6539,7 @@
         <x:v>矩阵单选（每行5点）</x:v>
       </x:c>
       <x:c r="E13" s="22" t="str">
-        <x:v>行：数值可靠性；方法覆盖；速度；GPU/HPC；易安装；GUI；Python/API；许可成本；支持；开源可审计；现有流程兼容。列：完全不重要–非常重要；不了解</x:v>
+        <x:v>行：数值可靠性；方法覆盖；速度；GPU/HPC；易安装；GUI；Python/API；默认设置透明度；许可成本；支持；开源可审计；现有流程兼容。列：完全不重要–非常重要；不了解</x:v>
       </x:c>
       <x:c r="F13" s="22" t="str">
         <x:v>是</x:v>
@@ -6566,7 +6566,7 @@
         <x:v>多选（最多3项）</x:v>
       </x:c>
       <x:c r="E14" s="22" t="str">
-        <x:v>同行评议软件论文；独立跨程序基准；与实验吻合；公开源代码；自动测试；长期版本稳定；实验室/同事惯例；厂商支持；高引用量；大型用户群；其他</x:v>
+        <x:v>同行评议软件论文；独立跨程序基准；公开输入、版本、容差和原始输出的可复现协议；与实验吻合；公开源代码；自动测试；长期版本稳定；实验室/同事惯例；厂商支持；高引用量；大型用户群；其他</x:v>
       </x:c>
       <x:c r="F14" s="22" t="str">
         <x:v>是</x:v>
@@ -6614,25 +6614,25 @@
         <x:v>可信度</x:v>
       </x:c>
       <x:c r="C16" s="22" t="str">
-        <x:v>过去12个月您使用哪些程序或方法做过交叉核验？</x:v>
+        <x:v>过去12个月，您对重要计算结果实际采取过哪些核验动作？</x:v>
       </x:c>
       <x:c r="D16" s="22" t="str">
         <x:v>多选</x:v>
       </x:c>
       <x:c r="E16" s="22" t="str">
-        <x:v>Gaussian；ORCA；PySCF；Psi4；Q-Chem；Molpro/CFOUR；VASP/Quantum ESPRESSO/CP2K；自写实现；实验数据；公开基准集；其他；未做过</x:v>
+        <x:v>使用另一计算程序复算；与公开基准集比较；与实验数据比较；加密积分网格；检查SCF稳定性或更换初猜；提高基组或检查基组/ECP版本；收紧收敛阈值；检查频率/驻点性质；记录并复核程序特定默认值；对实验比较加入ZPVE/热力学/相对论等必要校正；复核原始输出而非只看可视化；其他；未做过</x:v>
       </x:c>
       <x:c r="F16" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="G16" s="22" t="str">
-        <x:v>Q11=从不者可直接选择“未做过”</x:v>
+        <x:v>“未做过”与其他选项互斥</x:v>
       </x:c>
       <x:c r="H16" s="22" t="str">
-        <x:v>核验对象</x:v>
+        <x:v>实际核验动作</x:v>
       </x:c>
       <x:c r="I16" s="30" t="str">
-        <x:v>crosscheck_methods</x:v>
+        <x:v>verification_actions_12m</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
@@ -6649,7 +6649,7 @@
         <x:v>多选（最多3项）</x:v>
       </x:c>
       <x:c r="E17" s="22" t="str">
-        <x:v>误判轨道/相位；误判密度或静电势；坐标/单位错误；周期边界错误；图像无法复现；批量任务静默失败；论文图或汇报返工；结论受影响；仅影响美观；其他</x:v>
+        <x:v>误判轨道/相位；误判密度或静电势；网格/采样不足造成场值或等值面偏差；坐标/单位错误；周期边界错误；图像无法复现；批量任务静默失败；论文图或汇报返工；结论受影响；仅影响美观；其他</x:v>
       </x:c>
       <x:c r="F17" s="22" t="str">
         <x:v>是</x:v>
@@ -6811,7 +6811,7 @@
         <x:v>多选（最多3项）</x:v>
       </x:c>
       <x:c r="E23" s="22" t="str">
-        <x:v>从计算结果提取/转换格式；单位/坐标/周期边界；选择等值面阈值；交互传递函数/裁剪；正负相位；多个态/轨道及跨帧一致性；批量处理；动画；材质/灯光；复现参数；超大网格内存；软件兼容；其他；无明显痛点</x:v>
+        <x:v>从计算结果提取/转换格式；单位/坐标/周期边界；选择等值面阈值；交互传递函数/裁剪；正负相位；多个态/轨道及跨帧一致性；网格评估速度；大规模时间序列的存储/传输；批量处理；动画；材质/灯光；复现参数；超大网格内存；软件兼容；其他；无明显痛点</x:v>
       </x:c>
       <x:c r="F23" s="22" t="str">
         <x:v>是</x:v>
@@ -6838,7 +6838,7 @@
         <x:v>多选（最多6项）</x:v>
       </x:c>
       <x:c r="E24" s="22" t="str">
-        <x:v>源程序及版本；方法/泛函；基组/ECP/赝势；程序特定关键字及非默认设置；电荷与自旋；网格原点和三个轴向量；单位；场类型及轨道/态索引；等值面/传递函数参数；原始文件哈希；转换工具版本；完整输入/输出或计算记录链接；其他</x:v>
+        <x:v>源程序、版本和运行平台；方法/泛函及实现版本；基组/ECP/赝势的版本或来源；程序特定关键字、默认值覆盖和积分网格；电荷与自旋；网格原点和三个轴向量；单位；场类型及轨道/态索引；等值面/传递函数参数；原始文件哈希；转换工具版本；完整输入/输出或计算记录链接；其他</x:v>
       </x:c>
       <x:c r="F24" s="22" t="str">
         <x:v>是</x:v>
@@ -6892,7 +6892,7 @@
         <x:v>多选（最多5项）</x:v>
       </x:c>
       <x:c r="E26" s="22" t="str">
-        <x:v>多格式输入；保留完整计算元数据；保留程序特定控制并报告适配器能力；数值校验报告；一键Blender场景；交互等值面/体渲染/裁剪；正负轨道叶分离；周期单胞/超胞；多帧动画；NTO/差分密度；大网格稀疏VDB；批处理；Python API；GUI；自动图注；原始文件哈希归档</x:v>
+        <x:v>多格式输入；保留完整计算元数据；保留程序特定控制并报告适配器能力；数值校验报告；一键Blender场景；交互等值面/体渲染/裁剪；正负轨道叶分离；周期单胞/超胞；多帧动画与跨帧态/相位一致性；NTO/差分密度；大网格稀疏VDB；批处理；Python API；GUI；自动图注；原始文件哈希归档</x:v>
       </x:c>
       <x:c r="F26" s="22" t="str">
         <x:v>是</x:v>
@@ -6973,7 +6973,7 @@
         <x:v>单选</x:v>
       </x:c>
       <x:c r="E29" s="22" t="str">
-        <x:v>不支持现有文件格式；难以安装；需要额外编程/脚本经验；缺少GUI；无法在HPC/离线环境运行；缺少科学验证；处理大文件太慢；不能批量自动化；许可证/合规问题；团队已有稳定方案；没有足够需求；其他</x:v>
+        <x:v>不支持现有文件格式；难以安装；需要额外编程/脚本经验；缺少GUI；无法在HPC/离线环境运行；需要特定GPU/驱动环境；缺少科学验证；处理大文件太慢；不能批量自动化；许可证/合规问题；团队已有稳定方案；没有足够需求；其他</x:v>
       </x:c>
       <x:c r="F29" s="22" t="str">
         <x:v>是</x:v>
@@ -7056,7 +7056,7 @@
         <x:v>多选</x:v>
       </x:c>
       <x:c r="E32" s="108" t="str">
-        <x:v>安装/Windows；收敛；默认设置不清；性能；缺少方法/性质；文档；GUI；输出后处理；团队不熟悉；许可/合规；无明显障碍；其他</x:v>
+        <x:v>安装/Windows；收敛；默认设置或数值协议不清；性能；GPU/驱动环境；缺少方法/性质；文档；GUI；输出后处理；团队不熟悉；许可/合规；无明显障碍；其他</x:v>
       </x:c>
       <x:c r="F32" s="108" t="str">
         <x:v>是</x:v>
@@ -7085,7 +7085,7 @@
         <x:v>多选（最多3项）</x:v>
       </x:c>
       <x:c r="E33" s="108" t="str">
-        <x:v>不了解；主程序已满足；缺少GUI；团队标准不是PySCF；担心认可度；担心数值一致性；安装/Windows；缺少所需方法；性能；商业支持；其他</x:v>
+        <x:v>不了解；主程序已满足；缺少GUI；需要Python/脚本经验；团队标准不是PySCF；担心认可度；担心数值一致性；安装/Windows；GPU/驱动环境；缺少所需方法；性能；商业支持；其他</x:v>
       </x:c>
       <x:c r="F33" s="108" t="str">
         <x:v>是</x:v>
@@ -7139,7 +7139,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc4f1b89327e4369"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f8a04a5e7574233"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7880,7 +7880,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red6389d6ee454492"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2774d95689654506"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>